<commit_message>
Mettre à jour les correspondances édito et resynchroniser les affectations finales.
Le tableau s'appuie sur les scripts montés et la sélection finale des experts ; le site édito, suivi et guides est régénéré en conséquence.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/site/selection_finale_videos_expertise.xlsx
+++ b/site/selection_finale_videos_expertise.xlsx
@@ -681,135 +681,135 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Stephanie Sano</t>
+          <t>Arielle Santé</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>UVSQ (Université de Versailles Saint-Quentin-en-Yvelines)</t>
+          <t>IncubAlliance</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Experte UVSQ (Université de Versailles Saint-Quentin-en-Yvelines)</t>
+          <t>Entrepreneuriat deeptech / incubation</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>E8</t>
+          <t>E7</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 8</t>
+          <t>Vidéo Expert 7</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Brevetabilite, secret, savoir-faire, logiciel, preuve et confidentialite.</t>
+          <t>Premier contact, rôle du charge de valorisation et informations utiles pour examiner un résultat.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Stanislas De Lapasse</t>
+          <t>Stephanie Sano</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>INPI</t>
+          <t>UVSQ (Université de Versailles Saint-Quentin-en-Yvelines)</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Propriété industrielle / INPI</t>
+          <t>Experte UVSQ (Université de Versailles Saint-Quentin-en-Yvelines)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>E9</t>
+          <t>E8</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 9</t>
+          <t>Vidéo Expert 8</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Barriere à l'entree, pouvoir de negociation, credibilite et articulation avec le modele de valorisation.</t>
+          <t>Brevetabilite, secret, savoir-faire, logiciel, preuve et confidentialite.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Stanislas De Lapasse</t>
+          <t>Arielle Santé</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>INPI</t>
+          <t>IncubAlliance</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Propriété industrielle / INPI</t>
+          <t>Entrepreneuriat deeptech / incubation</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>E10</t>
+          <t>E8</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 10</t>
+          <t>Vidéo Expert 8</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Licence, création, co-développement, partenariat et criteres de choix.</t>
+          <t>Brevetabilite, secret, savoir-faire, logiciel, preuve et confidentialite.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Virginia Branco</t>
+          <t>Stanislas De Lapasse</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>ENS Paris-Saclay</t>
+          <t>INPI</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Appui recherche-innovation / transfert technologique</t>
+          <t>Propriété industrielle / INPI</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>E11</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 11</t>
+          <t>Vidéo Expert 9</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Licence exclusive ou non, cession, contrat de collaboration, copropriete et principes de negociation.</t>
+          <t>Barriere à l'entree, pouvoir de negociation, credibilite et articulation avec le modele de valorisation.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Soizic Lefeuvre</t>
+          <t>Antoine Latreille</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -819,56 +819,56 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Partenariat et valorisation / droit contrats et PI</t>
+          <t>Droit de l'innovation / propriété industrielle</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>E12</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 12</t>
+          <t>Vidéo Expert 9</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Étapes, sélection, investissement, jalons et accompagnement.</t>
+          <t>Barriere à l'entree, pouvoir de negociation, credibilite et articulation avec le modele de valorisation.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Fatoumata Aonon</t>
+          <t>Stanislas De Lapasse</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>CNRS</t>
+          <t>INPI</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Valorisation recherche / accompagnement projets</t>
+          <t>Propriété industrielle / INPI</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>E13</t>
+          <t>E10</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 13</t>
+          <t>Vidéo Expert 10</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Coaching, réseau, formation, confrontation, équipe et préparation de la création.</t>
+          <t>Licence, création, co-développement, partenariat et criteres de choix.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -890,150 +890,150 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>E13BIS</t>
+          <t>E10</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 13 BIS</t>
+          <t>Vidéo Expert 10</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Design spot, fablab, pole de competitivite, OTT, etc.</t>
+          <t>Licence, création, co-développement, partenariat et criteres de choix.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Yoann Montenot</t>
+          <t>Virginia Branco</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Université Paris-Saclay</t>
+          <t>ENS Paris-Saclay</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Design d'innovation / Design Spot Paris-Saclay</t>
+          <t>Appui recherche-innovation / transfert technologique</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>E14</t>
+          <t>E11</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 14</t>
+          <t>Vidéo Expert 11</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Prématuration, maturation, aides non dilutives, concours, Bpifrance et financement prive.</t>
+          <t>Licence exclusive ou non, cession, contrat de collaboration, copropriete et principes de negociation.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Fatoumata Aonon</t>
+          <t>Soizic Lefeuvre</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>CNRS</t>
+          <t>Université Paris-Saclay</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Valorisation recherche / accompagnement projets</t>
+          <t>Partenariat et valorisation / droit contrats et PI</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>E15</t>
+          <t>E12</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 15</t>
+          <t>Vidéo Expert 12</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Dilution, retour attendu, rythme de croissance, gouvernance et compatibilite avec le projet.</t>
+          <t>Étapes, sélection, investissement, jalons et accompagnement.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Arielle Santé</t>
+          <t>Eneli Vino</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>IncubAlliance</t>
+          <t>CNRS</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Entrepreneuriat deeptech / incubation</t>
+          <t>Juridique PI / contrats / valorisation</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>E16</t>
+          <t>E12</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 16</t>
+          <t>Vidéo Expert 12</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Complémentarité, recrutement, rôle du CEO, du CSO et du CTO, et criteres humains.</t>
+          <t>Étapes, sélection, investissement, jalons et accompagnement.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Pascal Corbel</t>
+          <t>Fatoumata Aonon</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Université Paris-Saclay</t>
+          <t>CNRS</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Management innovation / PI / entrepreneuriat</t>
+          <t>Valorisation recherche / accompagnement projets</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>E17</t>
+          <t>E13BIS</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 17</t>
+          <t>Vidéo Expert 13 BIS</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Gouvernance, responsabilites, repartition du pouvoir, parts, pacte et prevention des conflits.</t>
+          <t>Design spot, fablab, pole de competitivite, OTT, etc.</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Antoine Latreille</t>
+          <t>Yoann Montenot</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1043,56 +1043,56 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Droit de l'innovation / propriété industrielle</t>
+          <t>Design d'innovation / Design Spot Paris-Saclay</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>E18</t>
+          <t>E14</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 18</t>
+          <t>Vidéo Expert 14</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Adapter le message selon l'utilisateur, le decideur, le partenaire ou l'investisseur.</t>
+          <t>Prématuration, maturation, aides non dilutives, concours, Bpifrance et financement prive.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Arielle Santé</t>
+          <t>Fatoumata Aonon</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>IncubAlliance</t>
+          <t>CNRS</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Entrepreneuriat deeptech / incubation</t>
+          <t>Valorisation recherche / accompagnement projets</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>E19</t>
+          <t>E16</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 19</t>
+          <t>Vidéo Expert 16</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Feedback, entrainement, mentorat et evolution de l'identite professionnelle.</t>
+          <t>Complémentarité, recrutement, rôle du CEO, du CSO et du CTO, et criteres humains.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1114,86 +1114,86 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>E20</t>
+          <t>E19</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 20</t>
+          <t>Vidéo Expert 19</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Double casquette, gouvernance, impartialite, evolution du metier de chercheur.</t>
+          <t>Feedback, entrainement, mentorat et evolution de l'identite professionnelle.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Bernard Yannou</t>
+          <t>Pascal Corbel</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>CentraleSupélec</t>
+          <t>Université Paris-Saclay</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Innovation / design engineering / deeptech</t>
+          <t>Management innovation / PI / entrepreneuriat</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>E21</t>
+          <t>E20</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 21</t>
+          <t>Vidéo Expert 20</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Temps, légitimité, entourage, doute ; incertitude, essais, pivot ; première action reversible.</t>
+          <t>Double casquette, gouvernance, impartialite, evolution du metier de chercheur.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Pascal Corbel</t>
+          <t>Bernard Yannou</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Université Paris-Saclay</t>
+          <t>CentraleSupélec</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Management innovation / PI / entrepreneuriat</t>
+          <t>Innovation / design engineering / deeptech</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>E22</t>
+          <t>E21</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 22</t>
+          <t>Vidéo Expert 21</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Objectifs partages, complémentarité, gouvernance, engagement, création et partage de valeur.</t>
+          <t>Temps, légitimité, entourage, doute ; incertitude, essais, pivot ; première action reversible.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Rémi Waché</t>
+          <t>Pascal Corbel</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1203,39 +1203,39 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Développement de partenariats recherche-industrie</t>
+          <t>Management innovation / PI / entrepreneuriat</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>E23</t>
+          <t>E22</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 23</t>
+          <t>Vidéo Expert 22</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Confidentialite, contrats, connaissances anterieures, résultats nouveaux, PI, publication et sortie du partenariat.</t>
+          <t>Objectifs partages, complémentarité, gouvernance, engagement, création et partage de valeur.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Eneli Vino</t>
+          <t>Rémi Waché</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>CNRS</t>
+          <t>Université Paris-Saclay</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Juridique PI / contrats / valorisation</t>
+          <t>Développement de partenariats recherche-industrie</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Onglet Tournage : planning des vidéos E, suivi plateau, Monica animatrice.
Monica Henao n’est pas une intervenante : intro/outro (objectifs, debrief, à retenir). Arielle = E13/E15/E18, Antoine = E17.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/site/selection_finale_videos_expertise.xlsx
+++ b/site/selection_finale_videos_expertise.xlsx
@@ -681,135 +681,135 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Arielle Santé</t>
+          <t>Stephanie Sano</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>IncubAlliance</t>
+          <t>UVSQ (Université de Versailles Saint-Quentin-en-Yvelines)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Entrepreneuriat deeptech / incubation</t>
+          <t>Experte UVSQ (Université de Versailles Saint-Quentin-en-Yvelines)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>E7</t>
+          <t>E8</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 7</t>
+          <t>Vidéo Expert 8</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Premier contact, rôle du charge de valorisation et informations utiles pour examiner un résultat.</t>
+          <t>Brevetabilite, secret, savoir-faire, logiciel, preuve et confidentialite.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Stephanie Sano</t>
+          <t>Stanislas De Lapasse</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>UVSQ (Université de Versailles Saint-Quentin-en-Yvelines)</t>
+          <t>INPI</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Experte UVSQ (Université de Versailles Saint-Quentin-en-Yvelines)</t>
+          <t>Propriété industrielle / INPI</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>E8</t>
+          <t>E9</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 8</t>
+          <t>Vidéo Expert 9</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Brevetabilite, secret, savoir-faire, logiciel, preuve et confidentialite.</t>
+          <t>Barriere à l'entree, pouvoir de negociation, credibilite et articulation avec le modele de valorisation.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Arielle Santé</t>
+          <t>Stanislas De Lapasse</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>IncubAlliance</t>
+          <t>INPI</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Entrepreneuriat deeptech / incubation</t>
+          <t>Propriété industrielle / INPI</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>E8</t>
+          <t>E10</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 8</t>
+          <t>Vidéo Expert 10</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Brevetabilite, secret, savoir-faire, logiciel, preuve et confidentialite.</t>
+          <t>Licence, création, co-développement, partenariat et criteres de choix.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Stanislas De Lapasse</t>
+          <t>Virginia Branco</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>INPI</t>
+          <t>ENS Paris-Saclay</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Propriété industrielle / INPI</t>
+          <t>Appui recherche-innovation / transfert technologique</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>E9</t>
+          <t>E11</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 9</t>
+          <t>Vidéo Expert 11</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Barriere à l'entree, pouvoir de negociation, credibilite et articulation avec le modele de valorisation.</t>
+          <t>Licence exclusive ou non, cession, contrat de collaboration, copropriete et principes de negociation.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Antoine Latreille</t>
+          <t>Soizic Lefeuvre</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -819,56 +819,56 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Droit de l'innovation / propriété industrielle</t>
+          <t>Partenariat et valorisation / droit contrats et PI</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>E9</t>
+          <t>E12</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 9</t>
+          <t>Vidéo Expert 12</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Barriere à l'entree, pouvoir de negociation, credibilite et articulation avec le modele de valorisation.</t>
+          <t>Étapes, sélection, investissement, jalons et accompagnement.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Stanislas De Lapasse</t>
+          <t>Fatoumata Aonon</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>INPI</t>
+          <t>CNRS</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Propriété industrielle / INPI</t>
+          <t>Valorisation recherche / accompagnement projets</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>E10</t>
+          <t>E13</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 10</t>
+          <t>Vidéo Expert 13</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Licence, création, co-développement, partenariat et criteres de choix.</t>
+          <t>Coaching, réseau, formation, confrontation, équipe et préparation de la création.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -890,118 +890,118 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>E10</t>
+          <t>E13BIS</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 10</t>
+          <t>Vidéo Expert 13 BIS</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Licence, création, co-développement, partenariat et criteres de choix.</t>
+          <t>Design spot, fablab, pole de competitivite, OTT, etc.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Virginia Branco</t>
+          <t>Yoann Montenot</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>ENS Paris-Saclay</t>
+          <t>Université Paris-Saclay</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Appui recherche-innovation / transfert technologique</t>
+          <t>Design d'innovation / Design Spot Paris-Saclay</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>E11</t>
+          <t>E14</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 11</t>
+          <t>Vidéo Expert 14</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Licence exclusive ou non, cession, contrat de collaboration, copropriete et principes de negociation.</t>
+          <t>Prématuration, maturation, aides non dilutives, concours, Bpifrance et financement prive.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Soizic Lefeuvre</t>
+          <t>Fatoumata Aonon</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Université Paris-Saclay</t>
+          <t>CNRS</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Partenariat et valorisation / droit contrats et PI</t>
+          <t>Valorisation recherche / accompagnement projets</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>E12</t>
+          <t>E15</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 12</t>
+          <t>Vidéo Expert 15</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Étapes, sélection, investissement, jalons et accompagnement.</t>
+          <t>Dilution, retour attendu, rythme de croissance, gouvernance et compatibilite avec le projet.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Fatoumata Aonon</t>
+          <t>Arielle Santé</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>CNRS</t>
+          <t>IncubAlliance</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Valorisation recherche / accompagnement projets</t>
+          <t>Entrepreneuriat deeptech / incubation</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>E13BIS</t>
+          <t>E16</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 13 BIS</t>
+          <t>Vidéo Expert 16</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Design spot, fablab, pole de competitivite, OTT, etc.</t>
+          <t>Complémentarité, recrutement, rôle du CEO, du CSO et du CTO, et criteres humains.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Yoann Montenot</t>
+          <t>Pascal Corbel</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1011,71 +1011,71 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Design d'innovation / Design Spot Paris-Saclay</t>
+          <t>Management innovation / PI / entrepreneuriat</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>E14</t>
+          <t>E17</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 14</t>
+          <t>Vidéo Expert 17</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Prématuration, maturation, aides non dilutives, concours, Bpifrance et financement prive.</t>
+          <t>Gouvernance, responsabilites, repartition du pouvoir, parts, pacte et prevention des conflits.</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Fatoumata Aonon</t>
+          <t>Antoine Latreille</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>CNRS</t>
+          <t>Université Paris-Saclay</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Valorisation recherche / accompagnement projets</t>
+          <t>Droit de l'innovation / propriété industrielle</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>E16</t>
+          <t>E18</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Vidéo Expert 16</t>
+          <t>Vidéo Expert 18</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Complémentarité, recrutement, rôle du CEO, du CSO et du CTO, et criteres humains.</t>
+          <t>Adapter le message selon l'utilisateur, le decideur, le partenaire ou l'investisseur.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Pascal Corbel</t>
+          <t>Arielle Santé</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Université Paris-Saclay</t>
+          <t>IncubAlliance</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Management innovation / PI / entrepreneuriat</t>
+          <t>Entrepreneuriat deeptech / incubation</t>
         </is>
       </c>
     </row>

</xml_diff>